<commit_message>
Added RF output for vowel, DGP3. DGP 3 seems ok now but let's see how SMPBART does. Added vowel dataset. MPBART code seems almost finished.
</commit_message>
<xml_diff>
--- a/output/rf_dgp3_output.xlsx
+++ b/output/rf_dgp3_output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5cac48941448979/Bureaublad/msc_thesis/thesis_code/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED8000FC760EF50AE26CEE07622EDE9E2BF2A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09CC7CD4-9FA3-4083-AC38-D8E76B3D4502}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED80050DF218D587FB2EC3C1637EDE9E2BF2A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00674C07-9A8A-4ED0-8002-23482F364A55}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misclassification_rates" sheetId="1" r:id="rId1"/>
@@ -378,52 +378,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.55000000000000004</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.56699999999999995</v>
+        <v>8.2000000000000003E-2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.53800000000000003</v>
+        <v>0.30499999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.57399999999999995</v>
+        <v>0.20300000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.58199999999999996</v>
+        <v>0.29199999999999998</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.59699999999999998</v>
+        <v>0.35499999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.58899999999999997</v>
+        <v>4.3999999999999997E-2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.60599999999999998</v>
+        <v>0.14799999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.59299999999999997</v>
+        <v>0.10100000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.55800000000000005</v>
+        <v>0.192</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -432,7 +432,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.57539999999999991</v>
+        <v>0.18759999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -441,7 +441,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>2.2011108306691139E-2</v>
+        <v>0.10270259111737262</v>
       </c>
     </row>
   </sheetData>
@@ -457,52 +457,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.68345306400000005</v>
+        <v>0.24677603200000001</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.684292232</v>
+        <v>0.15827772800000001</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.66959100800000004</v>
+        <v>0.39102856000000003</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.688593024</v>
+        <v>0.32035496000000002</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.70159588799999995</v>
+        <v>0.40880217600000002</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.69040416800000004</v>
+        <v>0.50856602399999995</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>0.68771003200000003</v>
+        <v>8.7515704E-2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.69576252000000005</v>
+        <v>0.25293551199999997</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.69603989600000005</v>
+        <v>0.19141724800000001</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.68553868799999995</v>
+        <v>0.28374508799999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -511,7 +511,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.68829805200000005</v>
+        <v>0.28494190319999996</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -520,7 +520,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>8.7840983944339271E-3</v>
+        <v>0.12653845776119838</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DGP3 might be OK now, went for different option; latent manifold dgp. MPBART works. Added MPBART output for DGP1.
</commit_message>
<xml_diff>
--- a/output/rf_dgp3_output.xlsx
+++ b/output/rf_dgp3_output.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5cac48941448979/Bureaublad/msc_thesis/thesis_code/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED80050DF218D587FB2EC3C1637EDE9E2BF2A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00674C07-9A8A-4ED0-8002-23482F364A55}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_42CED800BE17E9BFC8EEB6A160172FEDE9E2BF2B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D045B7D1-A4F2-40DF-A846-77DB31B1C395}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -378,52 +378,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.154</v>
+        <v>0.159</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>8.2000000000000003E-2</v>
+        <v>0.17299999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.30499999999999999</v>
+        <v>0.151</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.20300000000000001</v>
+        <v>0.16600000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.29199999999999998</v>
+        <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.35499999999999998</v>
+        <v>0.16500000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>4.3999999999999997E-2</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.14799999999999999</v>
+        <v>0.155</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.10100000000000001</v>
+        <v>0.17199999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.192</v>
+        <v>0.159</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -432,7 +432,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.18759999999999999</v>
+        <v>0.1651</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -441,7 +441,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>0.10270259111737262</v>
+        <v>9.0853973190193737E-3</v>
       </c>
     </row>
   </sheetData>
@@ -457,52 +457,52 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>0.24677603200000001</v>
+        <v>0.25785577599999998</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0.15827772800000001</v>
+        <v>0.27395160800000001</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>0.39102856000000003</v>
+        <v>0.263629856</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.32035496000000002</v>
+        <v>0.28767508000000003</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>0.40880217600000002</v>
+        <v>0.264279192</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>0.50856602399999995</v>
+        <v>0.27812805600000001</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>8.7515704E-2</v>
+        <v>0.29862819200000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>0.25293551199999997</v>
+        <v>0.25016095999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.19141724800000001</v>
+        <v>0.28178443199999997</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.28374508799999998</v>
+        <v>0.26508549599999998</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -511,7 +511,7 @@
       </c>
       <c r="B12">
         <f>AVERAGE(A1:A10)</f>
-        <v>0.28494190319999996</v>
+        <v>0.27211786479999994</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -520,7 +520,7 @@
       </c>
       <c r="B13">
         <f>_xlfn.STDEV.S(A1:A10)</f>
-        <v>0.12653845776119838</v>
+        <v>1.4705290309481946E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>